<commit_message>
feat(rooms): back-fill building/room_number for legacy localStorage + bake into example xlsx
Stale localStorage from before the structured-location refactor stored
rooms without campus/building/room_number. migrateRoomsEquipment now
takes the canonical rooms.json baseline and back-fills missing building/
room_number by id, with a regex fallback that extracts a number from the
room name (e.g. "Room 263 – PC Game Lab" → "263", "Studio 142" → "142").

Also ship the rooms deck inside example-schedule.xlsx so Resume from
Excel on the example hydrates room cards with full location data,
matching the chair-export shape.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/example-schedule.xlsx
+++ b/frontend/public/example-schedule.xlsx
@@ -1,17 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
+  <workbookProtection workbookPassword="1499" lockStructure="1" lockWindows="0"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Affinity First" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Time Pref First" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balanced" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_state" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cover First" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Time Pref First" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Balanced" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="_data_meta" sheetId="5" state="veryHidden" r:id="rId5"/>
+    <sheet name="_data_offerings" sheetId="6" state="veryHidden" r:id="rId6"/>
+    <sheet name="_data_rooms" sheetId="7" state="veryHidden" r:id="rId7"/>
+    <sheet name="_data_solver_results" sheetId="8" state="veryHidden" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -600,7 +603,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-04-18</t>
+          <t>Generated: 2026-04-24</t>
         </is>
       </c>
     </row>
@@ -646,7 +649,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Affinity First</t>
+          <t>Cover First</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -811,7 +814,7 @@
     <row r="1" ht="18" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
-          <t>Mode: Affinity First  |  Status: OPTIMAL  |  Score: 42</t>
+          <t>Mode: Cover First  |  Status: OPTIMAL  |  Score: 42</t>
         </is>
       </c>
     </row>
@@ -880,7 +883,7 @@
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C3" s="14" t="inlineStr">
@@ -931,7 +934,7 @@
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
@@ -999,7 +1002,7 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
@@ -1050,7 +1053,7 @@
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
@@ -1101,7 +1104,7 @@
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
@@ -1165,7 +1168,7 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C10" s="17" t="inlineStr">
@@ -1216,7 +1219,7 @@
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
@@ -1280,7 +1283,7 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
@@ -1331,7 +1334,7 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
@@ -1480,7 +1483,7 @@
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C3" s="14" t="inlineStr">
@@ -1531,7 +1534,7 @@
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
@@ -1599,7 +1602,7 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
@@ -1650,7 +1653,7 @@
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
@@ -1701,7 +1704,7 @@
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
@@ -1765,7 +1768,7 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C10" s="17" t="inlineStr">
@@ -1816,7 +1819,7 @@
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
@@ -1880,7 +1883,7 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
@@ -1931,7 +1934,7 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
@@ -2080,7 +2083,7 @@
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C3" s="14" t="inlineStr">
@@ -2131,7 +2134,7 @@
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
@@ -2199,7 +2202,7 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
@@ -2250,7 +2253,7 @@
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
@@ -2301,7 +2304,7 @@
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
@@ -2365,7 +2368,7 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C10" s="17" t="inlineStr">
@@ -2416,7 +2419,7 @@
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
@@ -2480,7 +2483,7 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
@@ -2531,7 +2534,7 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
@@ -2592,20 +2595,826 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>GAME_SCHEDULER_STATE_V1</t>
+          <t>marker</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>GAME_SCHEDULER_DATA_V2</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{"schema_version":1,"source":"example","exported_at":"2026-04-18T14:13:50.512835+00:00","quarter":"fall","year":2026,"solver_mode":"balanced","offerings":[{"catalog_id":"GAME_220","priority":"must_have","sections":1,"override_enrollment_cap":null,"override_room_type":null,"override_preferred_professors":null,"notes":null,"assigned_prof_id":"prof_dodson","assigned_room_id":"room_261","pinned":{"day_group":1,"time_slot":"8:00AM"}},{"catalog_id":"GAME_706","priority":"must_have","sections":1,"override_enrollment_cap":null,"override_room_type":null,"override_preferred_professors":null,"notes":null,"assigned_prof_id":"prof_lindsey","assigned_room_id":"room_261","pinned":{"day_group":2,"time_slot":"8:00AM"}},{"catalog_id":"GAME_256","priority":"must_have","sections":1,"override_enrollment_cap":null,"override_room_type":null,"override_preferred_professors":null,"notes":null,"assigned_prof_id":"prof_dodson","assigned_room_id":"room_261","pinned":{"day_group":1,"time_slot":"11:00AM"}},{"catalog_id":"GAME_360","priority":"must_have","sections":1,"override_enrollment_cap":null,"override_room_type":null,"override_preferred_professors":null,"notes":null,"assigned_prof_id":"prof_allen","assigned_room_id":"room_263","pinned":{"day_group":1,"time_slot":"11:00AM"}},{"catalog_id":"GAME_405","priority":"must_have","sections":1,"override_enrollment_cap":null,"override_room_type":null,"override_preferred_professors":null,"notes":null,"assigned_prof_id":"prof_avenali","assigned_room_id":"room_263","pinned":{"day_group":2,"time_slot":"11:00AM"}},{"catalog_id":"MOME_130","priority":"must_have","sections":1,"override_enrollment_cap":null,"override_room_type":null,"override_preferred_professors":null,"notes":null,"assigned_prof_id":"prof_spencer","assigned_room_id":"room_261","pinned":{"day_group":1,"time_slot":"2:00PM"}},{"catalog_id":"GAME_120","priority":"must_have","sections":1,"override_enrollment_cap":null,"override_room_type":null,"override_preferred_professors":null,"notes":null,"assigned_prof_id":"prof_allen","assigned_room_id":"room_263","pinned":{"day_group":2,"time_slot":"2:00PM"}},{"catalog_id":"AI_101","priority":"must_have","sections":1,"override_enrollment_cap":null,"override_room_type":null,"override_preferred_professors":null,"notes":null,"assigned_prof_id":"prof_imperato","assigned_room_id":"room_263","pinned":{"day_group":1,"time_slot":"5:00PM"}},{"catalog_id":"MOME_719","priority":"should_have","sections":1,"override_enrollment_cap":null,"override_room_type":null,"override_preferred_professors":null,"notes":null,"assigned_prof_id":"prof_maloney","assigned_room_id":"room_263","pinned":{"day_group":2,"time_slot":"5:00PM"}}],"solver_results":{"modes":[{"mode":"affinity_first","assignments":[{"catalog_id":"GAME_220","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_706","section_idx":0,"prof_id":"prof_lindsey","room_id":"room_261","day_group":2,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_256","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_360","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_405","section_idx":0,"prof_id":"prof_avenali","room_id":"room_263","day_group":2,"time_slot":"11:00AM","affinity_level":2,"time_pref":"morning"},{"catalog_id":"MOME_130","section_idx":0,"prof_id":"prof_spencer","room_id":"room_261","day_group":1,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"GAME_120","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":2,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"AI_101","section_idx":0,"prof_id":"prof_imperato","room_id":"room_263","day_group":1,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"},{"catalog_id":"MOME_719","section_idx":0,"prof_id":"prof_maloney","room_id":"room_263","day_group":2,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"}]},{"mode":"time_pref_first","assignments":[{"catalog_id":"GAME_220","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_706","section_idx":0,"prof_id":"prof_lindsey","room_id":"room_261","day_group":2,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_256","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_360","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_405","section_idx":0,"prof_id":"prof_avenali","room_id":"room_263","day_group":2,"time_slot":"11:00AM","affinity_level":2,"time_pref":"morning"},{"catalog_id":"MOME_130","section_idx":0,"prof_id":"prof_spencer","room_id":"room_261","day_group":1,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"GAME_120","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":2,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"AI_101","section_idx":0,"prof_id":"prof_imperato","room_id":"room_263","day_group":1,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"},{"catalog_id":"MOME_719","section_idx":0,"prof_id":"prof_maloney","room_id":"room_263","day_group":2,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"}]},{"mode":"balanced","assignments":[{"catalog_id":"GAME_220","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_706","section_idx":0,"prof_id":"prof_lindsey","room_id":"room_261","day_group":2,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_256","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_360","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_405","section_idx":0,"prof_id":"prof_avenali","room_id":"room_263","day_group":2,"time_slot":"11:00AM","affinity_level":2,"time_pref":"morning"},{"catalog_id":"MOME_130","section_idx":0,"prof_id":"prof_spencer","room_id":"room_261","day_group":1,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"GAME_120","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":2,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"AI_101","section_idx":0,"prof_id":"prof_imperato","room_id":"room_263","day_group":1,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"},{"catalog_id":"MOME_719","section_idx":0,"prof_id":"prof_maloney","room_id":"room_263","day_group":2,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"}]}]}}</t>
+          <t>schema_version</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>exported_at</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-04-24T21:25:46.901928+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>quarter</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>fall</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>solver_mode</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>balanced</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>catalog_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>sections</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>override_enrollment_cap</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>override_preferred_professors</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>assigned_prof_id</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>assigned_room_id</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>pinned</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GAME_220</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>prof_dodson</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>room_261</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>{"day_group":1,"time_slot":"8:00AM"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GAME_706</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>prof_lindsey</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>room_261</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>{"day_group":2,"time_slot":"8:00AM"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GAME_256</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>prof_dodson</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>room_261</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>{"day_group":1,"time_slot":"11:00AM"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GAME_360</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>prof_allen</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>room_263</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>{"day_group":1,"time_slot":"11:00AM"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GAME_405</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>prof_avenali</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>room_263</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>{"day_group":2,"time_slot":"11:00AM"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MOME_130</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>prof_spencer</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>room_261</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>{"day_group":1,"time_slot":"2:00PM"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GAME_120</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>prof_allen</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>room_263</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>{"day_group":2,"time_slot":"2:00PM"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AI_101</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>prof_imperato</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>room_263</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>{"day_group":1,"time_slot":"5:00PM"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MOME_719</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>should_have</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>prof_maloney</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>room_263</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>{"day_group":2,"time_slot":"5:00PM"}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>campus</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>building</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>room_number</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>station_count</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>display_count</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>capacity</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>equipment_tags</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>room_263</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Room 263 – PC Game Lab</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Savannah</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Montgomery Hall</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>263</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>PC game lab – 20 PCs, 2 displays</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>["lab","pc","pc_lab"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>room_261</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Room 261 – PC Game Lab</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Savannah</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Montgomery Hall</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>261</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>20</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>PC game lab – 20 PCs, 2 displays</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>["lab","pc","pc_lab"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>room_260</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Room 260 – Mac Design Lab</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Savannah</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Montgomery Hall</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>260</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>20</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Mac design lab – 20 Macs, 1 display. Motion media use.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>["lab","mac","mac_lab"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>room_259</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Room 259 – PC Design Lab</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Savannah</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Montgomery Hall</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>259</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>20</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>20</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>PC design lab – 20 PCs, 1 display. Verify full game software suite.</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>["lab","pc","pc_lab"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>room_258</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Room 258 – Teacher Station</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Savannah</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Montgomery Hall</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>258</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>24</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Teacher station only – 1 PC, 1 display. Lecture/discussion/Zoom use.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>["lecture_flex","pc"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>room_257</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Room 257 – Teacher Station</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Savannah</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Montgomery Hall</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>257</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>24</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Teacher station only – 1 PC, 1 display. Lecture/discussion/Zoom use.</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>["lecture_flex","pc"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>room_156</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Room 156 – Game Lab</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Savannah</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Montgomery Hall</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>156</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>10</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>20</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>The Game Lab – 10 PCs, 1 display, teacher station. Large studio for senior/thesis classes.</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>["lab","large_game_lab","lecture_flex","pc","pc_lab"]</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>{"modes":[{"mode":"cover_first","assignments":[{"catalog_id":"GAME_220","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_706","section_idx":0,"prof_id":"prof_lindsey","room_id":"room_261","day_group":2,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_256","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_360","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_405","section_idx":0,"prof_id":"prof_avenali","room_id":"room_263","day_group":2,"time_slot":"11:00AM","affinity_level":2,"time_pref":"morning"},{"catalog_id":"MOME_130","section_idx":0,"prof_id":"prof_spencer","room_id":"room_261","day_group":1,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"GAME_120","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":2,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"AI_101","section_idx":0,"prof_id":"prof_imperato","room_id":"room_263","day_group":1,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"},{"catalog_id":"MOME_719","section_idx":0,"prof_id":"prof_maloney","room_id":"room_263","day_group":2,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"}]},{"mode":"time_pref_first","assignments":[{"catalog_id":"GAME_220","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_706","section_idx":0,"prof_id":"prof_lindsey","room_id":"room_261","day_group":2,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_256","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_360","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_405","section_idx":0,"prof_id":"prof_avenali","room_id":"room_263","day_group":2,"time_slot":"11:00AM","affinity_level":2,"time_pref":"morning"},{"catalog_id":"MOME_130","section_idx":0,"prof_id":"prof_spencer","room_id":"room_261","day_group":1,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"GAME_120","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":2,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"AI_101","section_idx":0,"prof_id":"prof_imperato","room_id":"room_263","day_group":1,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"},{"catalog_id":"MOME_719","section_idx":0,"prof_id":"prof_maloney","room_id":"room_263","day_group":2,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"}]},{"mode":"balanced","assignments":[{"catalog_id":"GAME_220","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_706","section_idx":0,"prof_id":"prof_lindsey","room_id":"room_261","day_group":2,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_256","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_360","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_405","section_idx":0,"prof_id":"prof_avenali","room_id":"room_263","day_group":2,"time_slot":"11:00AM","affinity_level":2,"time_pref":"morning"},{"catalog_id":"MOME_130","section_idx":0,"prof_id":"prof_spencer","room_id":"room_261","day_group":1,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"GAME_120","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":2,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"AI_101","section_idx":0,"prof_id":"prof_imperato","room_id":"room_263","day_group":1,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"},{"catalog_id":"MOME_719","section_idx":0,"prof_id":"prof_maloney","room_id":"room_263","day_group":2,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"}]}]}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(rooms): back-fill building/room_number for legacy localStorage + bake into example xlsx (#90)
Stale localStorage from before the structured-location refactor stored
rooms without campus/building/room_number. migrateRoomsEquipment now
takes the canonical rooms.json baseline and back-fills missing building/
room_number by id, with a regex fallback that extracts a number from the
room name (e.g. "Room 263 – PC Game Lab" → "263", "Studio 142" → "142").

Also ship the rooms deck inside example-schedule.xlsx so Resume from
Excel on the example hydrates room cards with full location data,
matching the chair-export shape.

Co-authored-by: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/example-schedule.xlsx
+++ b/frontend/public/example-schedule.xlsx
@@ -1,17 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
+  <workbookProtection workbookPassword="1499" lockStructure="1" lockWindows="0"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Affinity First" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Time Pref First" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balanced" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_state" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cover First" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Time Pref First" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Balanced" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="_data_meta" sheetId="5" state="veryHidden" r:id="rId5"/>
+    <sheet name="_data_offerings" sheetId="6" state="veryHidden" r:id="rId6"/>
+    <sheet name="_data_rooms" sheetId="7" state="veryHidden" r:id="rId7"/>
+    <sheet name="_data_solver_results" sheetId="8" state="veryHidden" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -600,7 +603,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-04-18</t>
+          <t>Generated: 2026-04-24</t>
         </is>
       </c>
     </row>
@@ -646,7 +649,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Affinity First</t>
+          <t>Cover First</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -811,7 +814,7 @@
     <row r="1" ht="18" customHeight="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
-          <t>Mode: Affinity First  |  Status: OPTIMAL  |  Score: 42</t>
+          <t>Mode: Cover First  |  Status: OPTIMAL  |  Score: 42</t>
         </is>
       </c>
     </row>
@@ -880,7 +883,7 @@
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C3" s="14" t="inlineStr">
@@ -931,7 +934,7 @@
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
@@ -999,7 +1002,7 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
@@ -1050,7 +1053,7 @@
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
@@ -1101,7 +1104,7 @@
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
@@ -1165,7 +1168,7 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C10" s="17" t="inlineStr">
@@ -1216,7 +1219,7 @@
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
@@ -1280,7 +1283,7 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
@@ -1331,7 +1334,7 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
@@ -1480,7 +1483,7 @@
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C3" s="14" t="inlineStr">
@@ -1531,7 +1534,7 @@
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
@@ -1599,7 +1602,7 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
@@ -1650,7 +1653,7 @@
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
@@ -1701,7 +1704,7 @@
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
@@ -1765,7 +1768,7 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C10" s="17" t="inlineStr">
@@ -1816,7 +1819,7 @@
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
@@ -1880,7 +1883,7 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
@@ -1931,7 +1934,7 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
@@ -2080,7 +2083,7 @@
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C3" s="14" t="inlineStr">
@@ -2131,7 +2134,7 @@
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
@@ -2199,7 +2202,7 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
@@ -2250,7 +2253,7 @@
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
@@ -2301,7 +2304,7 @@
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
@@ -2365,7 +2368,7 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C10" s="17" t="inlineStr">
@@ -2416,7 +2419,7 @@
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
@@ -2480,7 +2483,7 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>Mon/Wed</t>
+          <t>Monday/Wednesday</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
@@ -2531,7 +2534,7 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>Tue/Thu</t>
+          <t>Tuesday/Thursday</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
@@ -2592,20 +2595,826 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>GAME_SCHEDULER_STATE_V1</t>
+          <t>marker</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>GAME_SCHEDULER_DATA_V2</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{"schema_version":1,"source":"example","exported_at":"2026-04-18T14:13:50.512835+00:00","quarter":"fall","year":2026,"solver_mode":"balanced","offerings":[{"catalog_id":"GAME_220","priority":"must_have","sections":1,"override_enrollment_cap":null,"override_room_type":null,"override_preferred_professors":null,"notes":null,"assigned_prof_id":"prof_dodson","assigned_room_id":"room_261","pinned":{"day_group":1,"time_slot":"8:00AM"}},{"catalog_id":"GAME_706","priority":"must_have","sections":1,"override_enrollment_cap":null,"override_room_type":null,"override_preferred_professors":null,"notes":null,"assigned_prof_id":"prof_lindsey","assigned_room_id":"room_261","pinned":{"day_group":2,"time_slot":"8:00AM"}},{"catalog_id":"GAME_256","priority":"must_have","sections":1,"override_enrollment_cap":null,"override_room_type":null,"override_preferred_professors":null,"notes":null,"assigned_prof_id":"prof_dodson","assigned_room_id":"room_261","pinned":{"day_group":1,"time_slot":"11:00AM"}},{"catalog_id":"GAME_360","priority":"must_have","sections":1,"override_enrollment_cap":null,"override_room_type":null,"override_preferred_professors":null,"notes":null,"assigned_prof_id":"prof_allen","assigned_room_id":"room_263","pinned":{"day_group":1,"time_slot":"11:00AM"}},{"catalog_id":"GAME_405","priority":"must_have","sections":1,"override_enrollment_cap":null,"override_room_type":null,"override_preferred_professors":null,"notes":null,"assigned_prof_id":"prof_avenali","assigned_room_id":"room_263","pinned":{"day_group":2,"time_slot":"11:00AM"}},{"catalog_id":"MOME_130","priority":"must_have","sections":1,"override_enrollment_cap":null,"override_room_type":null,"override_preferred_professors":null,"notes":null,"assigned_prof_id":"prof_spencer","assigned_room_id":"room_261","pinned":{"day_group":1,"time_slot":"2:00PM"}},{"catalog_id":"GAME_120","priority":"must_have","sections":1,"override_enrollment_cap":null,"override_room_type":null,"override_preferred_professors":null,"notes":null,"assigned_prof_id":"prof_allen","assigned_room_id":"room_263","pinned":{"day_group":2,"time_slot":"2:00PM"}},{"catalog_id":"AI_101","priority":"must_have","sections":1,"override_enrollment_cap":null,"override_room_type":null,"override_preferred_professors":null,"notes":null,"assigned_prof_id":"prof_imperato","assigned_room_id":"room_263","pinned":{"day_group":1,"time_slot":"5:00PM"}},{"catalog_id":"MOME_719","priority":"should_have","sections":1,"override_enrollment_cap":null,"override_room_type":null,"override_preferred_professors":null,"notes":null,"assigned_prof_id":"prof_maloney","assigned_room_id":"room_263","pinned":{"day_group":2,"time_slot":"5:00PM"}}],"solver_results":{"modes":[{"mode":"affinity_first","assignments":[{"catalog_id":"GAME_220","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_706","section_idx":0,"prof_id":"prof_lindsey","room_id":"room_261","day_group":2,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_256","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_360","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_405","section_idx":0,"prof_id":"prof_avenali","room_id":"room_263","day_group":2,"time_slot":"11:00AM","affinity_level":2,"time_pref":"morning"},{"catalog_id":"MOME_130","section_idx":0,"prof_id":"prof_spencer","room_id":"room_261","day_group":1,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"GAME_120","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":2,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"AI_101","section_idx":0,"prof_id":"prof_imperato","room_id":"room_263","day_group":1,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"},{"catalog_id":"MOME_719","section_idx":0,"prof_id":"prof_maloney","room_id":"room_263","day_group":2,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"}]},{"mode":"time_pref_first","assignments":[{"catalog_id":"GAME_220","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_706","section_idx":0,"prof_id":"prof_lindsey","room_id":"room_261","day_group":2,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_256","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_360","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_405","section_idx":0,"prof_id":"prof_avenali","room_id":"room_263","day_group":2,"time_slot":"11:00AM","affinity_level":2,"time_pref":"morning"},{"catalog_id":"MOME_130","section_idx":0,"prof_id":"prof_spencer","room_id":"room_261","day_group":1,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"GAME_120","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":2,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"AI_101","section_idx":0,"prof_id":"prof_imperato","room_id":"room_263","day_group":1,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"},{"catalog_id":"MOME_719","section_idx":0,"prof_id":"prof_maloney","room_id":"room_263","day_group":2,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"}]},{"mode":"balanced","assignments":[{"catalog_id":"GAME_220","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_706","section_idx":0,"prof_id":"prof_lindsey","room_id":"room_261","day_group":2,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_256","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_360","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_405","section_idx":0,"prof_id":"prof_avenali","room_id":"room_263","day_group":2,"time_slot":"11:00AM","affinity_level":2,"time_pref":"morning"},{"catalog_id":"MOME_130","section_idx":0,"prof_id":"prof_spencer","room_id":"room_261","day_group":1,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"GAME_120","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":2,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"AI_101","section_idx":0,"prof_id":"prof_imperato","room_id":"room_263","day_group":1,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"},{"catalog_id":"MOME_719","section_idx":0,"prof_id":"prof_maloney","room_id":"room_263","day_group":2,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"}]}]}}</t>
+          <t>schema_version</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>exported_at</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-04-24T21:25:46.901928+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>quarter</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>fall</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>solver_mode</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>balanced</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>catalog_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>sections</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>override_enrollment_cap</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>override_preferred_professors</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>assigned_prof_id</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>assigned_room_id</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>pinned</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GAME_220</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>prof_dodson</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>room_261</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>{"day_group":1,"time_slot":"8:00AM"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GAME_706</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>prof_lindsey</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>room_261</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>{"day_group":2,"time_slot":"8:00AM"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GAME_256</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>prof_dodson</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>room_261</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>{"day_group":1,"time_slot":"11:00AM"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GAME_360</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>prof_allen</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>room_263</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>{"day_group":1,"time_slot":"11:00AM"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GAME_405</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>prof_avenali</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>room_263</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>{"day_group":2,"time_slot":"11:00AM"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MOME_130</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>prof_spencer</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>room_261</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>{"day_group":1,"time_slot":"2:00PM"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GAME_120</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>prof_allen</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>room_263</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>{"day_group":2,"time_slot":"2:00PM"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AI_101</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>prof_imperato</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>room_263</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>{"day_group":1,"time_slot":"5:00PM"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MOME_719</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>should_have</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>prof_maloney</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>room_263</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>{"day_group":2,"time_slot":"5:00PM"}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>campus</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>building</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>room_number</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>station_count</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>display_count</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>capacity</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>equipment_tags</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>room_263</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Room 263 – PC Game Lab</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Savannah</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Montgomery Hall</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>263</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>PC game lab – 20 PCs, 2 displays</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>["lab","pc","pc_lab"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>room_261</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Room 261 – PC Game Lab</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Savannah</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Montgomery Hall</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>261</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>20</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>PC game lab – 20 PCs, 2 displays</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>["lab","pc","pc_lab"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>room_260</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Room 260 – Mac Design Lab</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Savannah</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Montgomery Hall</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>260</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>20</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Mac design lab – 20 Macs, 1 display. Motion media use.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>["lab","mac","mac_lab"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>room_259</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Room 259 – PC Design Lab</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Savannah</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Montgomery Hall</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>259</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>20</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>20</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>PC design lab – 20 PCs, 1 display. Verify full game software suite.</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>["lab","pc","pc_lab"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>room_258</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Room 258 – Teacher Station</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Savannah</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Montgomery Hall</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>258</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>24</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Teacher station only – 1 PC, 1 display. Lecture/discussion/Zoom use.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>["lecture_flex","pc"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>room_257</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Room 257 – Teacher Station</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Savannah</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Montgomery Hall</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>257</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>24</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Teacher station only – 1 PC, 1 display. Lecture/discussion/Zoom use.</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>["lecture_flex","pc"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>room_156</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Room 156 – Game Lab</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Savannah</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Montgomery Hall</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>156</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>10</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>20</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>The Game Lab – 10 PCs, 1 display, teacher station. Large studio for senior/thesis classes.</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>["lab","large_game_lab","lecture_flex","pc","pc_lab"]</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>{"modes":[{"mode":"cover_first","assignments":[{"catalog_id":"GAME_220","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_706","section_idx":0,"prof_id":"prof_lindsey","room_id":"room_261","day_group":2,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_256","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_360","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_405","section_idx":0,"prof_id":"prof_avenali","room_id":"room_263","day_group":2,"time_slot":"11:00AM","affinity_level":2,"time_pref":"morning"},{"catalog_id":"MOME_130","section_idx":0,"prof_id":"prof_spencer","room_id":"room_261","day_group":1,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"GAME_120","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":2,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"AI_101","section_idx":0,"prof_id":"prof_imperato","room_id":"room_263","day_group":1,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"},{"catalog_id":"MOME_719","section_idx":0,"prof_id":"prof_maloney","room_id":"room_263","day_group":2,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"}]},{"mode":"time_pref_first","assignments":[{"catalog_id":"GAME_220","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_706","section_idx":0,"prof_id":"prof_lindsey","room_id":"room_261","day_group":2,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_256","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_360","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_405","section_idx":0,"prof_id":"prof_avenali","room_id":"room_263","day_group":2,"time_slot":"11:00AM","affinity_level":2,"time_pref":"morning"},{"catalog_id":"MOME_130","section_idx":0,"prof_id":"prof_spencer","room_id":"room_261","day_group":1,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"GAME_120","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":2,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"AI_101","section_idx":0,"prof_id":"prof_imperato","room_id":"room_263","day_group":1,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"},{"catalog_id":"MOME_719","section_idx":0,"prof_id":"prof_maloney","room_id":"room_263","day_group":2,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"}]},{"mode":"balanced","assignments":[{"catalog_id":"GAME_220","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_706","section_idx":0,"prof_id":"prof_lindsey","room_id":"room_261","day_group":2,"time_slot":"8:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_256","section_idx":0,"prof_id":"prof_dodson","room_id":"room_261","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_360","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":1,"time_slot":"11:00AM","affinity_level":1,"time_pref":"morning"},{"catalog_id":"GAME_405","section_idx":0,"prof_id":"prof_avenali","room_id":"room_263","day_group":2,"time_slot":"11:00AM","affinity_level":2,"time_pref":"morning"},{"catalog_id":"MOME_130","section_idx":0,"prof_id":"prof_spencer","room_id":"room_261","day_group":1,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"GAME_120","section_idx":0,"prof_id":"prof_allen","room_id":"room_263","day_group":2,"time_slot":"2:00PM","affinity_level":1,"time_pref":"afternoon"},{"catalog_id":"AI_101","section_idx":0,"prof_id":"prof_imperato","room_id":"room_263","day_group":1,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"},{"catalog_id":"MOME_719","section_idx":0,"prof_id":"prof_maloney","room_id":"room_263","day_group":2,"time_slot":"5:00PM","affinity_level":2,"time_pref":"afternoon_evening"}]}]}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(rooms): default all rooms to Atlanta / FORTY FIVE
Tim teaches 100% of his GAME classes at Atlanta / FORTY FIVE, so
every place the app says "default campus" now means Atlanta:

- data/rooms.json: 7 rooms switched from Savannah / Montgomery Hall
- example xlsx regenerated with the new defaults
- CAMPUSES enum reordered so Atlanta is first in the <select>
- addRoom() seeds campus=Atlanta, building=FORTY FIVE
- migrateRoomsEquipment + RoomCard + collectBuildingsByCampus
  fallbacks flipped from "Savannah" → "Atlanta"

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/example-schedule.xlsx
+++ b/frontend/public/example-schedule.xlsx
@@ -2628,7 +2628,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-04-24T21:25:46.901928+00:00</t>
+          <t>2026-04-24T21:48:50.801744+00:00</t>
         </is>
       </c>
     </row>
@@ -3088,12 +3088,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Montgomery Hall</t>
+          <t>FORTY FIVE</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -3134,12 +3134,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Montgomery Hall</t>
+          <t>FORTY FIVE</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -3180,12 +3180,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Montgomery Hall</t>
+          <t>FORTY FIVE</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -3226,12 +3226,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Montgomery Hall</t>
+          <t>FORTY FIVE</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -3272,12 +3272,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Montgomery Hall</t>
+          <t>FORTY FIVE</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -3318,12 +3318,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Montgomery Hall</t>
+          <t>FORTY FIVE</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -3364,12 +3364,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Montgomery Hall</t>
+          <t>FORTY FIVE</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">

</xml_diff>

<commit_message>
feat(rooms): default all rooms to Atlanta / FORTY FIVE (#92)
Tim teaches 100% of his GAME classes at Atlanta / FORTY FIVE, so
every place the app says "default campus" now means Atlanta:

- data/rooms.json: 7 rooms switched from Savannah / Montgomery Hall
- example xlsx regenerated with the new defaults
- CAMPUSES enum reordered so Atlanta is first in the <select>
- addRoom() seeds campus=Atlanta, building=FORTY FIVE
- migrateRoomsEquipment + RoomCard + collectBuildingsByCampus
  fallbacks flipped from "Savannah" → "Atlanta"

Co-authored-by: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/example-schedule.xlsx
+++ b/frontend/public/example-schedule.xlsx
@@ -2628,7 +2628,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-04-24T21:25:46.901928+00:00</t>
+          <t>2026-04-24T21:48:50.801744+00:00</t>
         </is>
       </c>
     </row>
@@ -3088,12 +3088,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Montgomery Hall</t>
+          <t>FORTY FIVE</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -3134,12 +3134,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Montgomery Hall</t>
+          <t>FORTY FIVE</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -3180,12 +3180,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Montgomery Hall</t>
+          <t>FORTY FIVE</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -3226,12 +3226,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Montgomery Hall</t>
+          <t>FORTY FIVE</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -3272,12 +3272,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Montgomery Hall</t>
+          <t>FORTY FIVE</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -3318,12 +3318,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Montgomery Hall</t>
+          <t>FORTY FIVE</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -3364,12 +3364,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Montgomery Hall</t>
+          <t>FORTY FIVE</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">

</xml_diff>